<commit_message>
Add source-document coverage check to the review
Verified the network paths are genuinely unreachable from this environment
(no mounts, host does not resolve, no smb client) rather than assuming it.

Cross-checked instead what the итоговый actually cites: 306 rows carry a
"(Файл: …)" reference covering 18 documents, and 7 of them are absent from
the 18 paths provided — АР.1 (99 rows), ПЗУ (56), ПОС (36), ТХ.2 (11), ТХ.3,
АК.1 and an unreadable HCOM code. That leaves 209 of the 306 referenced rows
with no source document to check against.

Also records that those 18 documents are cited under 45 different filename
spellings — АР.1 alone appears nine ways, and one reference reads nb2.pdf in
Latin instead of ПБ2.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U31bfjDxnG5ui2CtvwHcoC
</commit_message>
<xml_diff>
--- a/revue/РЕВЬЮ_итогового_файла.xlsx
+++ b/revue/РЕВЬЮ_итогового_файла.xlsx
@@ -8,10 +8,11 @@
   </bookViews>
   <sheets>
     <sheet name="Итог ревью" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Разделы и деньги" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Расхождения с ВОР" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Опечатки" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Формулы" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Документы и пути" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Разделы и деньги" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Расхождения с ВОР" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Опечатки" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Формулы" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +25,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="#,##0;[Red](#,##0);-"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -67,6 +68,16 @@
       <name val="Arial"/>
       <b val="1"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="6">
@@ -123,7 +134,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -188,6 +199,40 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -823,6 +868,1281 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F62"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="66" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="26" t="inlineStr">
+        <is>
+          <t>НА КАКИЕ ИСХОДНЫЕ ДОКУМЕНТЫ ССЫЛАЕТСЯ ИТОГОВЫЙ И ЧТО ИЗ ЭТОГО ПРИСЛАНО</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="27" t="inlineStr">
+        <is>
+          <t>Проверено по колонке «Примечание» листа «Спецификация»: 306 позиций содержат ссылку «(Файл: …)». Пути \\fs\share\… технически недоступны — сетевых монтирований нет, хост fs не резолвится, smb-клиента в системе нет.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Документ</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Что это</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Позиций ссылается</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Написаний имени файла</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Прислан?</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>Строки в «Спецификации»</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="28" t="inlineStr">
+        <is>
+          <t>АР.1</t>
+        </is>
+      </c>
+      <c r="B5" s="29" t="inlineStr">
+        <is>
+          <t>Архитектурные решения</t>
+        </is>
+      </c>
+      <c r="C5" s="28" t="n">
+        <v>99</v>
+      </c>
+      <c r="D5" s="28" t="n">
+        <v>9</v>
+      </c>
+      <c r="E5" s="28" t="inlineStr">
+        <is>
+          <t>НЕТ — нужен</t>
+        </is>
+      </c>
+      <c r="F5" s="29" t="inlineStr">
+        <is>
+          <t>4126, 4127, 4128, 4129, 4130, 4131, 4132, 4133, 4134, 4135, 4136, 4137, 4138, 4139, 4140, 4141, 4142, 4146, 4147, 4148, 4149, 4150, 4151, 4152, 4153, 4154 …</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="28" t="inlineStr">
+        <is>
+          <t>ПЗУ</t>
+        </is>
+      </c>
+      <c r="B6" s="29" t="inlineStr">
+        <is>
+          <t>Планировка земельного участка</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="n">
+        <v>56</v>
+      </c>
+      <c r="D6" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="E6" s="28" t="inlineStr">
+        <is>
+          <t>НЕТ — нужен</t>
+        </is>
+      </c>
+      <c r="F6" s="29" t="inlineStr">
+        <is>
+          <t>3, 16, 4238, 4239, 4240, 4241, 4242, 4243, 4244, 4245, 4246, 4247, 4248, 4249, 4250, 4251, 4252, 4253, 4254, 4255, 4256, 4257, 4258, 4259, 4261, 4262 …</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="28" t="inlineStr">
+        <is>
+          <t>ПОС</t>
+        </is>
+      </c>
+      <c r="B7" s="29" t="inlineStr">
+        <is>
+          <t>Проект организации строительства</t>
+        </is>
+      </c>
+      <c r="C7" s="28" t="n">
+        <v>36</v>
+      </c>
+      <c r="D7" s="28" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="28" t="inlineStr">
+        <is>
+          <t>НЕТ — нужен</t>
+        </is>
+      </c>
+      <c r="F7" s="29" t="inlineStr">
+        <is>
+          <t>6, 7, 8, 9, 10, 11, 12, 13, 14, 4295, 4296, 4297, 4298, 4299, 4300, 4301, 4302, 4303, 4304, 4305, 4306, 4307, 4308, 4309, 4310, 4311 …</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="30" t="inlineStr">
+        <is>
+          <t>КР</t>
+        </is>
+      </c>
+      <c r="B8" s="31" t="inlineStr">
+        <is>
+          <t>Конструктивные решения</t>
+        </is>
+      </c>
+      <c r="C8" s="30" t="n">
+        <v>29</v>
+      </c>
+      <c r="D8" s="30" t="n">
+        <v>4</v>
+      </c>
+      <c r="E8" s="30" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="F8" s="31" t="inlineStr">
+        <is>
+          <t>4, 4096, 4097, 4098, 4099, 4100, 4101, 4102, 4103, 4104, 4105, 4106, 4107, 4108, 4109, 4110, 4111, 4112, 4113, 4114, 4116, 4117, 4118, 4119, 4120, 4121 …</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="30" t="inlineStr">
+        <is>
+          <t>ИОС.2.1</t>
+        </is>
+      </c>
+      <c r="B9" s="31" t="inlineStr">
+        <is>
+          <t>Водоснабжение</t>
+        </is>
+      </c>
+      <c r="C9" s="30" t="n">
+        <v>25</v>
+      </c>
+      <c r="D9" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" s="30" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="F9" s="31" t="inlineStr">
+        <is>
+          <t>384, 385, 386, 387, 388, 389, 390, 391, 392, 393, 394, 395, 396, 397, 398, 399, 400, 401, 402, 403, 404, 405, 406, 407, 408</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="30" t="inlineStr">
+        <is>
+          <t>ИОС.4.4</t>
+        </is>
+      </c>
+      <c r="B10" s="31" t="inlineStr">
+        <is>
+          <t>Наружные сети теплоснабжения</t>
+        </is>
+      </c>
+      <c r="C10" s="30" t="n">
+        <v>15</v>
+      </c>
+      <c r="D10" s="30" t="n">
+        <v>6</v>
+      </c>
+      <c r="E10" s="30" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="F10" s="31" t="inlineStr">
+        <is>
+          <t>15, 1515, 1516, 4322, 4323, 4324, 4325, 4326, 4327, 4328, 4329, 4330, 4331, 4332, 4333</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="28" t="inlineStr">
+        <is>
+          <t>ТХ.2</t>
+        </is>
+      </c>
+      <c r="B11" s="29" t="inlineStr">
+        <is>
+          <t>Оборудование, мебель и инвентарь</t>
+        </is>
+      </c>
+      <c r="C11" s="28" t="n">
+        <v>11</v>
+      </c>
+      <c r="D11" s="28" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" s="28" t="inlineStr">
+        <is>
+          <t>НЕТ — нужен</t>
+        </is>
+      </c>
+      <c r="F11" s="29" t="inlineStr">
+        <is>
+          <t>4229, 4230, 4231, 4233, 4234, 4235, 4236, 4334, 4335, 4336, 4337</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="30" t="inlineStr">
+        <is>
+          <t>ИОС.3.1</t>
+        </is>
+      </c>
+      <c r="B12" s="31" t="inlineStr">
+        <is>
+          <t>Канализация</t>
+        </is>
+      </c>
+      <c r="C12" s="30" t="n">
+        <v>9</v>
+      </c>
+      <c r="D12" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" s="30" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="F12" s="31" t="inlineStr">
+        <is>
+          <t>423, 424, 425, 426, 427, 428, 429, 430, 431</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="30" t="inlineStr">
+        <is>
+          <t>ИОС.4.2</t>
+        </is>
+      </c>
+      <c r="B13" s="31" t="inlineStr">
+        <is>
+          <t>Вентиляция и кондиционирование</t>
+        </is>
+      </c>
+      <c r="C13" s="30" t="n">
+        <v>6</v>
+      </c>
+      <c r="D13" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="30" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="F13" s="31" t="inlineStr">
+        <is>
+          <t>1226, 1227, 1228, 1229, 1230, 1231</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="30" t="inlineStr">
+        <is>
+          <t>ИОС.5.1</t>
+        </is>
+      </c>
+      <c r="B14" s="31" t="inlineStr">
+        <is>
+          <t>Сети связи</t>
+        </is>
+      </c>
+      <c r="C14" s="30" t="n">
+        <v>6</v>
+      </c>
+      <c r="D14" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="30" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="F14" s="31" t="inlineStr">
+        <is>
+          <t>1894, 1895, 1896, 1897, 1898, 1899</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="30" t="inlineStr">
+        <is>
+          <t>ПБ2</t>
+        </is>
+      </c>
+      <c r="B15" s="31" t="inlineStr">
+        <is>
+          <t>Пожарная сигнализация</t>
+        </is>
+      </c>
+      <c r="C15" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="D15" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" s="30" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="F15" s="31" t="inlineStr">
+        <is>
+          <t>2487, 2488, 2489</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="28" t="inlineStr">
+        <is>
+          <t>ТХ.3</t>
+        </is>
+      </c>
+      <c r="B16" s="29" t="inlineStr">
+        <is>
+          <t>Технология (часть 3)</t>
+        </is>
+      </c>
+      <c r="C16" s="28" t="n">
+        <v>3</v>
+      </c>
+      <c r="D16" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="28" t="inlineStr">
+        <is>
+          <t>НЕТ — нужен</t>
+        </is>
+      </c>
+      <c r="F16" s="29" t="inlineStr">
+        <is>
+          <t>4090, 4091, 4092</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="28" t="inlineStr">
+        <is>
+          <t>АК.1</t>
+        </is>
+      </c>
+      <c r="B17" s="29" t="inlineStr">
+        <is>
+          <t>Архитектурные конструкции</t>
+        </is>
+      </c>
+      <c r="C17" s="28" t="n">
+        <v>3</v>
+      </c>
+      <c r="D17" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="28" t="inlineStr">
+        <is>
+          <t>НЕТ — нужен</t>
+        </is>
+      </c>
+      <c r="F17" s="29" t="inlineStr">
+        <is>
+          <t>4143, 4144, 4145</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="30" t="inlineStr">
+        <is>
+          <t>ИОС.1.5</t>
+        </is>
+      </c>
+      <c r="B18" s="31" t="inlineStr">
+        <is>
+          <t>Внешние сети электроснабжения</t>
+        </is>
+      </c>
+      <c r="C18" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="30" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="F18" s="31" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="30" t="inlineStr">
+        <is>
+          <t>ИОС.1.4</t>
+        </is>
+      </c>
+      <c r="B19" s="31" t="inlineStr">
+        <is>
+          <t>Наружное электроосвещение</t>
+        </is>
+      </c>
+      <c r="C19" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="30" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="F19" s="31" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="30" t="inlineStr">
+        <is>
+          <t>ИОС.3.2</t>
+        </is>
+      </c>
+      <c r="B20" s="31" t="inlineStr">
+        <is>
+          <t>Дренаж</t>
+        </is>
+      </c>
+      <c r="C20" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="30" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="F20" s="31" t="inlineStr">
+        <is>
+          <t>439</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="30" t="inlineStr">
+        <is>
+          <t>ИОС.4.3</t>
+        </is>
+      </c>
+      <c r="B21" s="31" t="inlineStr">
+        <is>
+          <t>ИТП</t>
+        </is>
+      </c>
+      <c r="C21" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="30" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="F21" s="31" t="inlineStr">
+        <is>
+          <t>558</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="28" t="inlineStr">
+        <is>
+          <t>HCOM</t>
+        </is>
+      </c>
+      <c r="B22" s="29" t="inlineStr">
+        <is>
+          <t>не расшифровывается — код битый</t>
+        </is>
+      </c>
+      <c r="C22" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="28" t="inlineStr">
+        <is>
+          <t>НЕТ — нужен</t>
+        </is>
+      </c>
+      <c r="F22" s="29" t="inlineStr">
+        <is>
+          <t>1514</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="32" t="n"/>
+      <c r="B23" s="16" t="inlineStr">
+        <is>
+          <t>ИТОГО позиций со ссылкой на файл</t>
+        </is>
+      </c>
+      <c r="C23" s="33">
+        <f>SUM(C5:C22)</f>
+        <v/>
+      </c>
+      <c r="D23" s="32" t="n"/>
+      <c r="E23" s="32" t="n"/>
+      <c r="F23" s="34" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="32" t="n"/>
+      <c r="B24" s="34" t="n"/>
+      <c r="C24" s="32" t="n"/>
+      <c r="D24" s="32" t="n"/>
+      <c r="E24" s="32" t="n"/>
+      <c r="F24" s="34" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="35" t="inlineStr">
+        <is>
+          <t>ОДИН ДОКУМЕНТ — РАЗНЫЕ ИМЕНА ФАЙЛА В ПРИМЕЧАНИЯХ</t>
+        </is>
+      </c>
+      <c r="B25" s="34" t="n"/>
+      <c r="C25" s="32" t="n"/>
+      <c r="D25" s="32" t="n"/>
+      <c r="E25" s="32" t="n"/>
+      <c r="F25" s="34" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="36" t="inlineStr">
+        <is>
+          <t>Документ</t>
+        </is>
+      </c>
+      <c r="B26" s="24" t="inlineStr">
+        <is>
+          <t>Как записано имя файла</t>
+        </is>
+      </c>
+      <c r="C26" s="36" t="inlineStr">
+        <is>
+          <t>Позиций</t>
+        </is>
+      </c>
+      <c r="D26" s="32" t="n"/>
+      <c r="E26" s="32" t="n"/>
+      <c r="F26" s="34" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="32" t="inlineStr">
+        <is>
+          <t>ПЗУ</t>
+        </is>
+      </c>
+      <c r="B27" s="37" t="inlineStr">
+        <is>
+          <t>03- 01 07.21П-ПЗУ .pdf</t>
+        </is>
+      </c>
+      <c r="C27" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D27" s="32" t="n"/>
+      <c r="E27" s="32" t="n"/>
+      <c r="F27" s="34" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="32" t="inlineStr">
+        <is>
+          <t>ПЗУ</t>
+        </is>
+      </c>
+      <c r="B28" s="37" t="inlineStr">
+        <is>
+          <t>03- 01_07.21П-ПЗУ .pdf</t>
+        </is>
+      </c>
+      <c r="C28" s="32" t="n">
+        <v>19</v>
+      </c>
+      <c r="D28" s="32" t="n"/>
+      <c r="E28" s="32" t="n"/>
+      <c r="F28" s="34" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="32" t="inlineStr">
+        <is>
+          <t>ПЗУ</t>
+        </is>
+      </c>
+      <c r="B29" s="37" t="inlineStr">
+        <is>
+          <t>03-01/07.21П-ПЗУ .pdf</t>
+        </is>
+      </c>
+      <c r="C29" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="D29" s="32" t="n"/>
+      <c r="E29" s="32" t="n"/>
+      <c r="F29" s="34" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="32" t="inlineStr">
+        <is>
+          <t>ПЗУ</t>
+        </is>
+      </c>
+      <c r="B30" s="37" t="inlineStr">
+        <is>
+          <t>03-01_07.21П- ПЗУ.pdf</t>
+        </is>
+      </c>
+      <c r="C30" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D30" s="32" t="n"/>
+      <c r="E30" s="32" t="n"/>
+      <c r="F30" s="34" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="32" t="inlineStr">
+        <is>
+          <t>ПЗУ</t>
+        </is>
+      </c>
+      <c r="B31" s="37" t="inlineStr">
+        <is>
+          <t>03-01_07.21П-ПЗУ .pdf</t>
+        </is>
+      </c>
+      <c r="C31" s="32" t="n">
+        <v>25</v>
+      </c>
+      <c r="D31" s="32" t="n"/>
+      <c r="E31" s="32" t="n"/>
+      <c r="F31" s="34" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="32" t="inlineStr">
+        <is>
+          <t>ПЗУ</t>
+        </is>
+      </c>
+      <c r="B32" s="37" t="inlineStr">
+        <is>
+          <t>03-01_07.21П-ПЗУ.pdf</t>
+        </is>
+      </c>
+      <c r="C32" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" s="32" t="n"/>
+      <c r="E32" s="32" t="n"/>
+      <c r="F32" s="34" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="32" t="inlineStr">
+        <is>
+          <t>КР</t>
+        </is>
+      </c>
+      <c r="B33" s="37" t="inlineStr">
+        <is>
+          <t>03- 01_07.21П-КР.pdf</t>
+        </is>
+      </c>
+      <c r="C33" s="32" t="n">
+        <v>11</v>
+      </c>
+      <c r="D33" s="32" t="n"/>
+      <c r="E33" s="32" t="n"/>
+      <c r="F33" s="34" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="32" t="inlineStr">
+        <is>
+          <t>КР</t>
+        </is>
+      </c>
+      <c r="B34" s="37" t="inlineStr">
+        <is>
+          <t>03-01/07.21П-КР.pdf</t>
+        </is>
+      </c>
+      <c r="C34" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" s="32" t="n"/>
+      <c r="E34" s="32" t="n"/>
+      <c r="F34" s="34" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="32" t="inlineStr">
+        <is>
+          <t>КР</t>
+        </is>
+      </c>
+      <c r="B35" s="37" t="inlineStr">
+        <is>
+          <t>03-01_07.21П-КР.pdf</t>
+        </is>
+      </c>
+      <c r="C35" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="D35" s="32" t="n"/>
+      <c r="E35" s="32" t="n"/>
+      <c r="F35" s="34" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="32" t="inlineStr">
+        <is>
+          <t>КР</t>
+        </is>
+      </c>
+      <c r="B36" s="29" t="inlineStr">
+        <is>
+          <t>Раздел_03- 0107.21П-КР!.pdf</t>
+        </is>
+      </c>
+      <c r="C36" s="32" t="n">
+        <v>9</v>
+      </c>
+      <c r="D36" s="32" t="n"/>
+      <c r="E36" s="32" t="n"/>
+      <c r="F36" s="34" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="32" t="inlineStr">
+        <is>
+          <t>ПОС</t>
+        </is>
+      </c>
+      <c r="B37" s="37" t="inlineStr">
+        <is>
+          <t>03-01/07.21П-ПОС.pdf</t>
+        </is>
+      </c>
+      <c r="C37" s="32" t="n">
+        <v>15</v>
+      </c>
+      <c r="D37" s="32" t="n"/>
+      <c r="E37" s="32" t="n"/>
+      <c r="F37" s="34" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="32" t="inlineStr">
+        <is>
+          <t>ПОС</t>
+        </is>
+      </c>
+      <c r="B38" s="37" t="inlineStr">
+        <is>
+          <t>03-01_07.21П-ПОС.pdf</t>
+        </is>
+      </c>
+      <c r="C38" s="32" t="n">
+        <v>21</v>
+      </c>
+      <c r="D38" s="32" t="n"/>
+      <c r="E38" s="32" t="n"/>
+      <c r="F38" s="34" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="32" t="inlineStr">
+        <is>
+          <t>ИОС.4.4</t>
+        </is>
+      </c>
+      <c r="B39" s="37" t="inlineStr">
+        <is>
+          <t>03- 01 07.21П-ИОС4.4.pdf</t>
+        </is>
+      </c>
+      <c r="C39" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D39" s="32" t="n"/>
+      <c r="E39" s="32" t="n"/>
+      <c r="F39" s="34" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="32" t="inlineStr">
+        <is>
+          <t>ИОС.4.4</t>
+        </is>
+      </c>
+      <c r="B40" s="37" t="inlineStr">
+        <is>
+          <t>03- 01_07.21П-ИОС4.4.pdf</t>
+        </is>
+      </c>
+      <c r="C40" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="D40" s="32" t="n"/>
+      <c r="E40" s="32" t="n"/>
+      <c r="F40" s="34" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="32" t="inlineStr">
+        <is>
+          <t>ИОС.4.4</t>
+        </is>
+      </c>
+      <c r="B41" s="37" t="inlineStr">
+        <is>
+          <t>03-01/07.21П-ИОС4.4.pdf</t>
+        </is>
+      </c>
+      <c r="C41" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D41" s="32" t="n"/>
+      <c r="E41" s="32" t="n"/>
+      <c r="F41" s="34" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="32" t="inlineStr">
+        <is>
+          <t>ИОС.4.4</t>
+        </is>
+      </c>
+      <c r="B42" s="37" t="inlineStr">
+        <is>
+          <t>03-01_07.21П- ИОС4.4.pdf</t>
+        </is>
+      </c>
+      <c r="C42" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" s="32" t="n"/>
+      <c r="E42" s="32" t="n"/>
+      <c r="F42" s="34" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="32" t="inlineStr">
+        <is>
+          <t>ИОС.4.4</t>
+        </is>
+      </c>
+      <c r="B43" s="37" t="inlineStr">
+        <is>
+          <t>03-01_07.21П-ИОС4.4.pdf</t>
+        </is>
+      </c>
+      <c r="C43" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" s="32" t="n"/>
+      <c r="E43" s="32" t="n"/>
+      <c r="F43" s="34" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="32" t="inlineStr">
+        <is>
+          <t>ИОС.4.4</t>
+        </is>
+      </c>
+      <c r="B44" s="29" t="inlineStr">
+        <is>
+          <t>03-01_07.21П-ИОС4.4.р#</t>
+        </is>
+      </c>
+      <c r="C44" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" s="32" t="n"/>
+      <c r="E44" s="32" t="n"/>
+      <c r="F44" s="34" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="32" t="inlineStr">
+        <is>
+          <t>ИОС.2.1</t>
+        </is>
+      </c>
+      <c r="B45" s="37" t="inlineStr">
+        <is>
+          <t>03- 01 07.21П-ИОС.2.pdf стр.: 1 2 3 4 5 6</t>
+        </is>
+      </c>
+      <c r="C45" s="32" t="n">
+        <v>14</v>
+      </c>
+      <c r="D45" s="32" t="n"/>
+      <c r="E45" s="32" t="n"/>
+      <c r="F45" s="34" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="32" t="inlineStr">
+        <is>
+          <t>ИОС.2.1</t>
+        </is>
+      </c>
+      <c r="B46" s="37" t="inlineStr">
+        <is>
+          <t>03- 01_07.21П-ИОС.2.pdf стр.: 1 2 3 4 5 6</t>
+        </is>
+      </c>
+      <c r="C46" s="32" t="n">
+        <v>11</v>
+      </c>
+      <c r="D46" s="32" t="n"/>
+      <c r="E46" s="32" t="n"/>
+      <c r="F46" s="34" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="32" t="inlineStr">
+        <is>
+          <t>ИОС.3.1</t>
+        </is>
+      </c>
+      <c r="B47" s="37" t="inlineStr">
+        <is>
+          <t>03-01/07.21П-ИОС3.1.pdf</t>
+        </is>
+      </c>
+      <c r="C47" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D47" s="32" t="n"/>
+      <c r="E47" s="32" t="n"/>
+      <c r="F47" s="34" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="32" t="inlineStr">
+        <is>
+          <t>ИОС.3.1</t>
+        </is>
+      </c>
+      <c r="B48" s="37" t="inlineStr">
+        <is>
+          <t>03-01_07.21П-ИОС3.1.pdf</t>
+        </is>
+      </c>
+      <c r="C48" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="D48" s="32" t="n"/>
+      <c r="E48" s="32" t="n"/>
+      <c r="F48" s="34" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="32" t="inlineStr">
+        <is>
+          <t>ПБ2</t>
+        </is>
+      </c>
+      <c r="B49" s="29" t="inlineStr">
+        <is>
+          <t>03-01_07.21П-nb2.pdf</t>
+        </is>
+      </c>
+      <c r="C49" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" s="32" t="n"/>
+      <c r="E49" s="32" t="n"/>
+      <c r="F49" s="34" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="32" t="inlineStr">
+        <is>
+          <t>ПБ2</t>
+        </is>
+      </c>
+      <c r="B50" s="37" t="inlineStr">
+        <is>
+          <t>03-01_07.21П-ПБ2.pdf</t>
+        </is>
+      </c>
+      <c r="C50" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D50" s="32" t="n"/>
+      <c r="E50" s="32" t="n"/>
+      <c r="F50" s="34" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="32" t="inlineStr">
+        <is>
+          <t>АР.1</t>
+        </is>
+      </c>
+      <c r="B51" s="37" t="inlineStr">
+        <is>
+          <t>03- 01 07.21П-АР.1.pdf</t>
+        </is>
+      </c>
+      <c r="C51" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="D51" s="32" t="n"/>
+      <c r="E51" s="32" t="n"/>
+      <c r="F51" s="34" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="32" t="inlineStr">
+        <is>
+          <t>АР.1</t>
+        </is>
+      </c>
+      <c r="B52" s="37" t="inlineStr">
+        <is>
+          <t>03- 01_07.21П-АР.1.pdf</t>
+        </is>
+      </c>
+      <c r="C52" s="32" t="n">
+        <v>23</v>
+      </c>
+      <c r="D52" s="32" t="n"/>
+      <c r="E52" s="32" t="n"/>
+      <c r="F52" s="34" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="32" t="inlineStr">
+        <is>
+          <t>АР.1</t>
+        </is>
+      </c>
+      <c r="B53" s="37" t="inlineStr">
+        <is>
+          <t>03-01_07.21П- АР.1.pdf</t>
+        </is>
+      </c>
+      <c r="C53" s="32" t="n">
+        <v>26</v>
+      </c>
+      <c r="D53" s="32" t="n"/>
+      <c r="E53" s="32" t="n"/>
+      <c r="F53" s="34" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="32" t="inlineStr">
+        <is>
+          <t>АР.1</t>
+        </is>
+      </c>
+      <c r="B54" s="37" t="inlineStr">
+        <is>
+          <t>03-01_07.21П- АР.1.pdf стр.: 14</t>
+        </is>
+      </c>
+      <c r="C54" s="32" t="n">
+        <v>16</v>
+      </c>
+      <c r="D54" s="32" t="n"/>
+      <c r="E54" s="32" t="n"/>
+      <c r="F54" s="34" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="32" t="inlineStr">
+        <is>
+          <t>АР.1</t>
+        </is>
+      </c>
+      <c r="B55" s="37" t="inlineStr">
+        <is>
+          <t>03-01_07.21П- АР.1.pdf стр.: 30</t>
+        </is>
+      </c>
+      <c r="C55" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="D55" s="32" t="n"/>
+      <c r="E55" s="32" t="n"/>
+      <c r="F55" s="34" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="32" t="inlineStr">
+        <is>
+          <t>АР.1</t>
+        </is>
+      </c>
+      <c r="B56" s="37" t="inlineStr">
+        <is>
+          <t>03-01_07.21П- АР.1.pdf стр.: 31</t>
+        </is>
+      </c>
+      <c r="C56" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="D56" s="32" t="n"/>
+      <c r="E56" s="32" t="n"/>
+      <c r="F56" s="34" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="32" t="inlineStr">
+        <is>
+          <t>АР.1</t>
+        </is>
+      </c>
+      <c r="B57" s="37" t="inlineStr">
+        <is>
+          <t>03-01_07.21П- АР.1.pdf стр.: 36</t>
+        </is>
+      </c>
+      <c r="C57" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D57" s="32" t="n"/>
+      <c r="E57" s="32" t="n"/>
+      <c r="F57" s="34" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="32" t="inlineStr">
+        <is>
+          <t>АР.1</t>
+        </is>
+      </c>
+      <c r="B58" s="37" t="inlineStr">
+        <is>
+          <t>03-01_07.21П- АР.1.pdf стр.: 41</t>
+        </is>
+      </c>
+      <c r="C58" s="32" t="n">
+        <v>9</v>
+      </c>
+      <c r="D58" s="32" t="n"/>
+      <c r="E58" s="32" t="n"/>
+      <c r="F58" s="34" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="32" t="inlineStr">
+        <is>
+          <t>АР.1</t>
+        </is>
+      </c>
+      <c r="B59" s="37" t="inlineStr">
+        <is>
+          <t>03-01_07.21П-АР.1.pdf</t>
+        </is>
+      </c>
+      <c r="C59" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D59" s="32" t="n"/>
+      <c r="E59" s="32" t="n"/>
+      <c r="F59" s="34" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="32" t="inlineStr">
+        <is>
+          <t>ТХ.2</t>
+        </is>
+      </c>
+      <c r="B60" s="37" t="inlineStr">
+        <is>
+          <t>03-01_07.21П-ТХ.2.pdf</t>
+        </is>
+      </c>
+      <c r="C60" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D60" s="32" t="n"/>
+      <c r="E60" s="32" t="n"/>
+      <c r="F60" s="34" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="32" t="inlineStr">
+        <is>
+          <t>ТХ.2</t>
+        </is>
+      </c>
+      <c r="B61" s="37" t="inlineStr">
+        <is>
+          <t>03-01_07.21П—ТХ.2.pdf</t>
+        </is>
+      </c>
+      <c r="C61" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D61" s="32" t="n"/>
+      <c r="E61" s="32" t="n"/>
+      <c r="F61" s="34" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="32" t="inlineStr">
+        <is>
+          <t>ТХ.2</t>
+        </is>
+      </c>
+      <c r="B62" s="29" t="inlineStr">
+        <is>
+          <t>Раздел_03-0107.21П ТХ.2!.pdf</t>
+        </is>
+      </c>
+      <c r="C62" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="D62" s="32" t="n"/>
+      <c r="E62" s="32" t="n"/>
+      <c r="F62" s="34" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1469,7 +2789,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1614,7 +2934,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2666,7 +3986,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>